<commit_message>
Add variable track offset segments and MPLUS2 fonts
- Add linear and arc track edge offset segment implementations with coverage for evaluation, compilation, and serialization
- Include MPLUS2 font assets for TextMeshPro usage
</commit_message>
<xml_diff>
--- a/Documentation/References/Stations.xlsx
+++ b/Documentation/References/Stations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yudai/Documents/Unity/Nakatetsu/Documentation/References/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{258BAA55-B75E-6B4F-8753-0D32CF3AF173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74783A3F-B2A3-F849-9AB0-2CAA3A117CDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="28200" xr2:uid="{E5B58C20-BF18-4243-BA31-F43A5F07EC81}"/>
+    <workbookView xWindow="-36000" yWindow="4480" windowWidth="36000" windowHeight="22600" activeTab="1" xr2:uid="{E5B58C20-BF18-4243-BA31-F43A5F07EC81}"/>
   </bookViews>
   <sheets>
     <sheet name="キロ程表" sheetId="1" r:id="rId1"/>
@@ -1406,13 +1406,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14435926-98F6-4441-8BF0-3B1866719C19}">
-  <dimension ref="B2:I32"/>
+  <dimension ref="B2:K32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>
   <cols>
     <col min="2" max="2" width="22.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9">
+    <row r="2" spans="2:11">
       <c r="B2" t="s">
         <v>14</v>
       </c>
@@ -1435,7 +1435,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="2:9">
+    <row r="3" spans="2:11">
       <c r="B3" t="s">
         <v>1</v>
       </c>
@@ -1458,7 +1458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="2:9">
+    <row r="4" spans="2:11">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -1481,7 +1481,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="5" spans="2:9">
+    <row r="5" spans="2:11">
       <c r="B5" t="s">
         <v>4</v>
       </c>
@@ -1503,8 +1503,11 @@
       <c r="I5">
         <v>2.1</v>
       </c>
-    </row>
-    <row r="6" spans="2:9">
+      <c r="K5">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11">
       <c r="B6" t="s">
         <v>5</v>
       </c>
@@ -1527,7 +1530,7 @@
         <v>3.2</v>
       </c>
     </row>
-    <row r="7" spans="2:9">
+    <row r="7" spans="2:11">
       <c r="B7" t="s">
         <v>6</v>
       </c>
@@ -1550,7 +1553,7 @@
         <v>3.9</v>
       </c>
     </row>
-    <row r="8" spans="2:9">
+    <row r="8" spans="2:11">
       <c r="B8" t="s">
         <v>7</v>
       </c>
@@ -1573,7 +1576,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="9" spans="2:9">
+    <row r="9" spans="2:11">
       <c r="B9" t="s">
         <v>8</v>
       </c>
@@ -1596,7 +1599,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="10" spans="2:9">
+    <row r="10" spans="2:11">
       <c r="B10" t="s">
         <v>9</v>
       </c>
@@ -1619,7 +1622,7 @@
         <v>7.4</v>
       </c>
     </row>
-    <row r="11" spans="2:9">
+    <row r="11" spans="2:11">
       <c r="B11" t="s">
         <v>10</v>
       </c>
@@ -1642,7 +1645,7 @@
         <v>8.4</v>
       </c>
     </row>
-    <row r="12" spans="2:9">
+    <row r="12" spans="2:11">
       <c r="B12" t="s">
         <v>11</v>
       </c>
@@ -1665,7 +1668,7 @@
         <v>9.6999999999999993</v>
       </c>
     </row>
-    <row r="13" spans="2:9">
+    <row r="13" spans="2:11">
       <c r="B13" t="s">
         <v>13</v>
       </c>
@@ -1688,7 +1691,7 @@
         <v>10.6</v>
       </c>
     </row>
-    <row r="14" spans="2:9">
+    <row r="14" spans="2:11">
       <c r="B14" t="s">
         <v>20</v>
       </c>
@@ -1711,7 +1714,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="15" spans="2:9">
+    <row r="15" spans="2:11">
       <c r="B15" t="s">
         <v>21</v>
       </c>
@@ -1734,7 +1737,7 @@
         <v>12.9</v>
       </c>
     </row>
-    <row r="16" spans="2:9">
+    <row r="16" spans="2:11">
       <c r="B16" t="s">
         <v>22</v>
       </c>

</xml_diff>

<commit_message>
Checkpoint W1-04 driving integration, Series10000 and TIMS displays
</commit_message>
<xml_diff>
--- a/Documentation/References/Stations.xlsx
+++ b/Documentation/References/Stations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yudai/Documents/Unity/Nakatetsu/Documentation/References/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74783A3F-B2A3-F849-9AB0-2CAA3A117CDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B88F258B-3ACF-8046-ADDD-C5A4A2A569B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-36000" yWindow="4480" windowWidth="36000" windowHeight="22600" activeTab="1" xr2:uid="{E5B58C20-BF18-4243-BA31-F43A5F07EC81}"/>
+    <workbookView xWindow="-36000" yWindow="4480" windowWidth="36000" windowHeight="22600" xr2:uid="{E5B58C20-BF18-4243-BA31-F43A5F07EC81}"/>
   </bookViews>
   <sheets>
     <sheet name="キロ程表" sheetId="1" r:id="rId1"/>
@@ -1406,13 +1406,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14435926-98F6-4441-8BF0-3B1866719C19}">
-  <dimension ref="B2:K32"/>
+  <dimension ref="B2:I32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>
   <cols>
     <col min="2" max="2" width="22.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11">
+    <row r="2" spans="2:9">
       <c r="B2" t="s">
         <v>14</v>
       </c>
@@ -1435,7 +1435,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="2:11">
+    <row r="3" spans="2:9">
       <c r="B3" t="s">
         <v>1</v>
       </c>
@@ -1458,7 +1458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="2:11">
+    <row r="4" spans="2:9">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -1481,7 +1481,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="5" spans="2:11">
+    <row r="5" spans="2:9">
       <c r="B5" t="s">
         <v>4</v>
       </c>
@@ -1503,11 +1503,8 @@
       <c r="I5">
         <v>2.1</v>
       </c>
-      <c r="K5">
-        <v>543</v>
-      </c>
-    </row>
-    <row r="6" spans="2:11">
+    </row>
+    <row r="6" spans="2:9">
       <c r="B6" t="s">
         <v>5</v>
       </c>
@@ -1530,7 +1527,7 @@
         <v>3.2</v>
       </c>
     </row>
-    <row r="7" spans="2:11">
+    <row r="7" spans="2:9">
       <c r="B7" t="s">
         <v>6</v>
       </c>
@@ -1553,7 +1550,7 @@
         <v>3.9</v>
       </c>
     </row>
-    <row r="8" spans="2:11">
+    <row r="8" spans="2:9">
       <c r="B8" t="s">
         <v>7</v>
       </c>
@@ -1576,7 +1573,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="9" spans="2:11">
+    <row r="9" spans="2:9">
       <c r="B9" t="s">
         <v>8</v>
       </c>
@@ -1599,7 +1596,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="10" spans="2:11">
+    <row r="10" spans="2:9">
       <c r="B10" t="s">
         <v>9</v>
       </c>
@@ -1622,7 +1619,7 @@
         <v>7.4</v>
       </c>
     </row>
-    <row r="11" spans="2:11">
+    <row r="11" spans="2:9">
       <c r="B11" t="s">
         <v>10</v>
       </c>
@@ -1645,7 +1642,7 @@
         <v>8.4</v>
       </c>
     </row>
-    <row r="12" spans="2:11">
+    <row r="12" spans="2:9">
       <c r="B12" t="s">
         <v>11</v>
       </c>
@@ -1668,7 +1665,7 @@
         <v>9.6999999999999993</v>
       </c>
     </row>
-    <row r="13" spans="2:11">
+    <row r="13" spans="2:9">
       <c r="B13" t="s">
         <v>13</v>
       </c>
@@ -1691,7 +1688,7 @@
         <v>10.6</v>
       </c>
     </row>
-    <row r="14" spans="2:11">
+    <row r="14" spans="2:9">
       <c r="B14" t="s">
         <v>20</v>
       </c>
@@ -1714,7 +1711,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="15" spans="2:11">
+    <row r="15" spans="2:9">
       <c r="B15" t="s">
         <v>21</v>
       </c>
@@ -1737,7 +1734,7 @@
         <v>12.9</v>
       </c>
     </row>
-    <row r="16" spans="2:11">
+    <row r="16" spans="2:9">
       <c r="B16" t="s">
         <v>22</v>
       </c>

</xml_diff>